<commit_message>
Refresh the TEST fleet reports with APM coverage
Adds the .NET agent columns and brings the counts up to date: 6 of 11 hosts
report infrastructure data, all 6 have Windows Services enabled, and 3 have
APM.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/IPAYOUT - Estado agente New Relic (TEST).xlsx
+++ b/reports/IPAYOUT - Estado agente New Relic (TEST).xlsx
@@ -56,13 +56,15 @@
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="46" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="4" max="4" width="48" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
     <col min="7" max="7" width="28" customWidth="1"/>
-    <col min="8" max="8" width="20" customWidth="1"/>
-    <col min="9" max="9" width="60" customWidth="1"/>
-    <col min="10" max="10" width="58" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
+    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="10" max="10" width="14" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="12" max="12" width="95" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -88,12 +90,12 @@
       </c>
       <c r="E1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Agente instalado</t>
+          <t xml:space="preserve">Agente infra</t>
         </is>
       </c>
       <c r="F1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Version del agente</t>
+          <t xml:space="preserve">Version infra</t>
         </is>
       </c>
       <c r="G1" t="inlineStr" s="1">
@@ -108,10 +110,20 @@
       </c>
       <c r="I1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Servicios IPS frenados</t>
+          <t xml:space="preserve">Agente .NET (APM)</t>
         </is>
       </c>
       <c r="J1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Version .NET</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Aplicaciones APM</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Observaciones</t>
         </is>
@@ -160,12 +172,22 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No reporta a New Relic - agente no instalado</t>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sin agente instalado</t>
         </is>
       </c>
     </row>
@@ -212,12 +234,22 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t xml:space="preserve">No reporta a New Relic - agente no instalado</t>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sin agente instalado</t>
         </is>
       </c>
     </row>
@@ -264,12 +296,22 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ips_deploymentservice</t>
+          <t xml:space="preserve">No</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IIS corriendo pero sin agente .NET: 0 transacciones en 30 dias</t>
         </is>
       </c>
     </row>
@@ -296,32 +338,42 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Si</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">1.80.3</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Si</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">292</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Si</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t xml:space="preserve">No reporta a New Relic - agente no instalado</t>
+          <t xml:space="preserve">10.54.0</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reporta con el nombre por defecto 'My Application' - quitar &lt;name&gt; de newrelic.config para que las apps tomen el nombre del app pool</t>
         </is>
       </c>
     </row>
@@ -368,10 +420,20 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t xml:space="preserve">ips_deploymentservice</t>
+          <t xml:space="preserve">Si</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10.54.0</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
         </is>
@@ -420,10 +482,20 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t xml:space="preserve">ips_deploymentservice</t>
+          <t xml:space="preserve">Si</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10.54.0</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
         </is>
@@ -472,12 +544,22 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t xml:space="preserve">No reporta a New Relic - agente no instalado</t>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sin agente instalado. Tambien necesita la integracion nri-mssql</t>
         </is>
       </c>
     </row>
@@ -524,12 +606,22 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t xml:space="preserve">No reporta a New Relic - agente no instalado</t>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sin agente instalado. Tambien necesita la integracion nri-mssql</t>
         </is>
       </c>
     </row>
@@ -576,12 +668,22 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t xml:space="preserve">ips_sendunsentachsservice, ips_svcorderprocessorservice, ips_recurringtransfersservice, ips_emailreceiverservice, ips_deploymentservice, ips_deletefilemanagerservice, ips_bai2reportsservice, ips_achreportservice</t>
+          <t xml:space="preserve">No</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t xml:space="preserve">8 servicios IPS frenados - requiere revision</t>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8 servicios IPS frenados. Necesita el agente .NET mas las variables CORECLR, porque los servicios no corren bajo IIS</t>
         </is>
       </c>
     </row>
@@ -628,12 +730,22 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reporta como UE1-TEST-SMT-A1 (nombre distinto, probablemente el mismo host)</t>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reporta como UE1-TEST-SMT-A1 (nombre distinto, probablemente el limite NetBIOS de 15 caracteres)</t>
         </is>
       </c>
     </row>
@@ -680,16 +792,26 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t xml:space="preserve">No reporta. La integracion Windows Services no aplica (Linux)</t>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Necesita el agente de Linux. Windows Services y el agente .NET no aplican</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J12"/>
+  <autoFilter ref="A1:L12"/>
 </worksheet>
 </file>
</xml_diff>